<commit_message>
chore: reset 現貨/在途 to 0 in inventory template
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/inventory-template.xlsx
+++ b/templates/inventory-template.xlsx
@@ -1258,7 +1258,7 @@
         <v>0</v>
       </c>
       <c r="P4" s="41" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="42" t="n"/>
     </row>
@@ -1310,7 +1310,7 @@
       <c r="M5" s="53" t="n"/>
       <c r="N5" s="39" t="n"/>
       <c r="O5" s="54" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="P5" s="55" t="n"/>
       <c r="Q5" s="42" t="n"/>
@@ -1362,7 +1362,7 @@
       <c r="M6" s="53" t="n"/>
       <c r="N6" s="39" t="n"/>
       <c r="O6" s="65" t="n">
-        <v>440</v>
+        <v>0</v>
       </c>
       <c r="P6" s="83" t="n"/>
       <c r="Q6" s="42" t="n"/>
@@ -1414,7 +1414,7 @@
       <c r="M7" s="53" t="n"/>
       <c r="N7" s="39" t="n"/>
       <c r="O7" s="65" t="n">
-        <v>290</v>
+        <v>0</v>
       </c>
       <c r="P7" s="83" t="n"/>
       <c r="Q7" s="42" t="n"/>
@@ -1466,7 +1466,7 @@
       <c r="M8" s="53" t="n"/>
       <c r="N8" s="39" t="n"/>
       <c r="O8" s="65" t="n">
-        <v>272</v>
+        <v>0</v>
       </c>
       <c r="P8" s="83" t="n"/>
       <c r="Q8" s="42" t="n"/>
@@ -1518,7 +1518,7 @@
       <c r="M9" s="53" t="n"/>
       <c r="N9" s="39" t="n"/>
       <c r="O9" s="65" t="n">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="P9" s="83" t="n"/>
       <c r="Q9" s="42" t="n"/>
@@ -1571,7 +1571,7 @@
       <c r="M10" s="53" t="n"/>
       <c r="N10" s="39" t="n"/>
       <c r="O10" s="65" t="n">
-        <v>156</v>
+        <v>0</v>
       </c>
       <c r="P10" s="83" t="n"/>
       <c r="Q10" s="42" t="n"/>
@@ -1624,10 +1624,10 @@
       <c r="M11" s="53" t="n"/>
       <c r="N11" s="81" t="n"/>
       <c r="O11" s="82" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="P11" s="83" t="n">
-        <v>144</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="42" t="n"/>
     </row>
@@ -1702,7 +1702,7 @@
       <c r="M13" s="53" t="n"/>
       <c r="N13" s="81" t="n"/>
       <c r="O13" s="65" t="n">
-        <v>368</v>
+        <v>0</v>
       </c>
       <c r="P13" s="83" t="n"/>
       <c r="Q13" s="42" t="n"/>
@@ -1754,10 +1754,10 @@
       <c r="M14" s="53" t="n"/>
       <c r="N14" s="81" t="n"/>
       <c r="O14" s="82" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="P14" s="83" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="Q14" s="42" t="n"/>
     </row>
@@ -1827,7 +1827,7 @@
       <c r="M16" s="53" t="n"/>
       <c r="N16" s="39" t="n"/>
       <c r="O16" s="65" t="n">
-        <v>504</v>
+        <v>0</v>
       </c>
       <c r="P16" s="83" t="n"/>
       <c r="Q16" s="42" t="n"/>
@@ -1880,7 +1880,7 @@
       <c r="M17" s="53" t="n"/>
       <c r="N17" s="39" t="n"/>
       <c r="O17" s="65" t="n">
-        <v>1104</v>
+        <v>0</v>
       </c>
       <c r="P17" s="83" t="n"/>
       <c r="Q17" s="42" t="n"/>
@@ -1933,10 +1933,10 @@
       <c r="M18" s="53" t="n"/>
       <c r="N18" s="39" t="n"/>
       <c r="O18" s="82" t="n">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="P18" s="83" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="42" t="n"/>
     </row>
@@ -1987,7 +1987,7 @@
       <c r="M19" s="53" t="n"/>
       <c r="N19" s="39" t="n"/>
       <c r="O19" s="65" t="n">
-        <v>272</v>
+        <v>0</v>
       </c>
       <c r="P19" s="83" t="n"/>
       <c r="Q19" s="42" t="n"/>
@@ -2039,7 +2039,7 @@
       <c r="M20" s="53" t="n"/>
       <c r="N20" s="39" t="n"/>
       <c r="O20" s="111" t="n">
-        <v>416</v>
+        <v>0</v>
       </c>
       <c r="P20" s="112" t="n"/>
       <c r="Q20" s="42" t="n"/>

</xml_diff>